<commit_message>
Cut the shoot to one surroundings frame and use the real FORUS logo
The client was right twice. Side A faces the traffic by definition, so its
general view already is the "view from the main flow" — a second frame from the
same spot was the same photograph under a different name. And the close-up of a
1.2x1.8 m poster adds nothing to the general view either.

Two of the four shot types in clause 5.2.1 remain: the general view, of which
102 of 106 already exist, and one surroundings frame per structure. 322 missing
shots become 58, and the sheet now spells out how to take that frame — stand
with your back to the panel, shoot the place, on a weekday when there is
traffic, because the frame answers "who will see this".

The header and footer carry the company's own mark from forus.by instead of a
letter tile; on the dark footer it sits on a white chip because the file has an
opaque light background. It also becomes the tab icon.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Задачи_Битрикс24_портал.xlsx
+++ b/Задачи_Битрикс24_портал.xlsx
@@ -432,7 +432,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">По каждой стороне — кадр со стороны потока; по конструкции — кадр окружения</t>
+          <t xml:space="preserve">По конструкции — один кадр окружения; общие планы уже загружены</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -506,7 +506,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">По каждой стороне — кадр со стороны потока; по конструкции — кадр окружения</t>
+          <t xml:space="preserve">По конструкции — один кадр окружения; общие планы уже загружены</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -543,7 +543,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">По каждой стороне — кадр со стороны потока; по конструкции — кадр окружения</t>
+          <t xml:space="preserve">По конструкции — один кадр окружения; общие планы уже загружены</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">По каждой стороне — кадр со стороны потока; по конструкции — кадр окружения</t>
+          <t xml:space="preserve">По конструкции — один кадр окружения; общие планы уже загружены</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Все 164 снимка из файла задания загружены</t>
+          <t xml:space="preserve">Все 58 снимков из файла задания загружены</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Remove the dismantled construction at Замковая, 4
The client confirms the structure is gone from the street. It is dropped from
the address programme: 51 constructions, 268 positions. Structure ids are left
as they are rather than renumbered, so the occupancy of every other position
stays where it was.

The designer's sheet loses three shots (55 now), and the two tasks that counted
constructions and shots are updated with it.

Also: the cover stats said "51 конструкций".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Задачи_Битрикс24_портал.xlsx
+++ b/Задачи_Битрикс24_портал.xlsx
@@ -338,7 +338,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Проверить на местности координаты 52 конструкций</t>
+          <t xml:space="preserve">Проверить на местности координаты 51 конструкции</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -358,7 +358,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Отмечено, где точка на карте стоит не на конструкции</t>
+          <t xml:space="preserve">Отмечено, где точка на карте стоит не на конструкции или конструкции больше нет</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Все 58 снимков из файла задания загружены</t>
+          <t xml:space="preserve">Все 55 снимков из файла задания загружены</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">

</xml_diff>